<commit_message>
data: Week 15 inventory + sales ETL complete - all brands processed
</commit_message>
<xml_diff>
--- a/data/raw/inventory/Week 15/White_Mulberry/Inventory Snapshot.xlsx
+++ b/data/raw/inventory/Week 15/White_Mulberry/Inventory Snapshot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 15\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B948A24B-DF61-48BA-923C-2742972BCB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02953720-CA53-4240-A7CB-F003D57B1BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -857,7 +857,47 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 6" xfId="1" xr:uid="{E5F241CE-C0FC-4730-81C9-F1901EB82A3C}"/>
   </cellStyles>
-  <dxfs count="134">
+  <dxfs count="135">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1128,36 +1168,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1222,26 +1232,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1326,6 +1316,236 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1390,236 +1610,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1664,46 +1654,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1788,6 +1738,206 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1832,206 +1982,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2044,6 +1994,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2156,6 +2116,96 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2170,46 +2220,6 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -7661,205 +7671,204 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L141" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A3:A27">
+    <cfRule type="duplicateValues" dxfId="134" priority="1001"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A27">
-    <cfRule type="duplicateValues" dxfId="133" priority="357"/>
-    <cfRule type="duplicateValues" dxfId="132" priority="358"/>
-    <cfRule type="duplicateValues" dxfId="131" priority="359"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="362"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="363" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="364" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="130" priority="360"/>
     <cfRule type="duplicateValues" dxfId="129" priority="361"/>
-    <cfRule type="duplicateValues" dxfId="128" priority="362"/>
-    <cfRule type="duplicateValues" dxfId="127" priority="363" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="126" priority="364" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="359"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="358"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="357"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A33:A43">
+    <cfRule type="duplicateValues" dxfId="125" priority="969"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A44:A66">
+    <cfRule type="duplicateValues" dxfId="124" priority="945"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="946"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A74:A84">
-    <cfRule type="duplicateValues" dxfId="125" priority="104"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="104"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A108:A132">
-    <cfRule type="duplicateValues" dxfId="124" priority="908"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="908"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A132">
-    <cfRule type="duplicateValues" dxfId="123" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="62"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="122" priority="856"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="856"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17 D5:D15">
+    <cfRule type="duplicateValues" dxfId="118" priority="976" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="975"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18:D27">
-    <cfRule type="duplicateValues" dxfId="121" priority="168"/>
-    <cfRule type="duplicateValues" dxfId="120" priority="169"/>
-    <cfRule type="duplicateValues" dxfId="119" priority="170"/>
-    <cfRule type="duplicateValues" dxfId="118" priority="171"/>
-    <cfRule type="duplicateValues" dxfId="117" priority="172"/>
-    <cfRule type="duplicateValues" dxfId="116" priority="173"/>
-    <cfRule type="duplicateValues" dxfId="115" priority="174" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="114" priority="175" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="168"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="172"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="170"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="169"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="174" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="173"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="175" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D29:D32">
+    <cfRule type="duplicateValues" dxfId="108" priority="951"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="950"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="956" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="955" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="954"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="953"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="952"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="949"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D75">
-    <cfRule type="duplicateValues" dxfId="113" priority="99" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="112" priority="100"/>
-    <cfRule type="duplicateValues" dxfId="111" priority="101" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="110" priority="102"/>
-    <cfRule type="duplicateValues" dxfId="109" priority="103" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="101" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="102"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="103" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="99" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="100"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D76">
-    <cfRule type="duplicateValues" dxfId="108" priority="94"/>
-    <cfRule type="duplicateValues" dxfId="107" priority="95"/>
-    <cfRule type="duplicateValues" dxfId="106" priority="96" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="105" priority="97" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="104" priority="98" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="95"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="96" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="97" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="98" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="94"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D77">
-    <cfRule type="duplicateValues" dxfId="103" priority="89"/>
-    <cfRule type="duplicateValues" dxfId="102" priority="90"/>
-    <cfRule type="duplicateValues" dxfId="101" priority="91" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="100" priority="92" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="99" priority="93" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="90"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="92" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="91" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="93" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D78">
-    <cfRule type="duplicateValues" dxfId="98" priority="88"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="88"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D82">
-    <cfRule type="duplicateValues" dxfId="97" priority="80"/>
-    <cfRule type="duplicateValues" dxfId="96" priority="81"/>
-    <cfRule type="duplicateValues" dxfId="95" priority="82"/>
-    <cfRule type="duplicateValues" dxfId="94" priority="83"/>
-    <cfRule type="duplicateValues" dxfId="93" priority="84"/>
-    <cfRule type="duplicateValues" dxfId="92" priority="85"/>
-    <cfRule type="duplicateValues" dxfId="91" priority="86" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="90" priority="87" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="85"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="84"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="87" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="86" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D83:D84">
-    <cfRule type="duplicateValues" dxfId="89" priority="72"/>
-    <cfRule type="duplicateValues" dxfId="88" priority="73"/>
-    <cfRule type="duplicateValues" dxfId="87" priority="74"/>
-    <cfRule type="duplicateValues" dxfId="86" priority="75"/>
-    <cfRule type="duplicateValues" dxfId="85" priority="76"/>
-    <cfRule type="duplicateValues" dxfId="84" priority="77"/>
-    <cfRule type="duplicateValues" dxfId="83" priority="78" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="82" priority="79" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="78" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="79" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D85:D107">
-    <cfRule type="duplicateValues" dxfId="81" priority="921"/>
-    <cfRule type="duplicateValues" dxfId="80" priority="922"/>
-    <cfRule type="duplicateValues" dxfId="79" priority="923"/>
-    <cfRule type="duplicateValues" dxfId="78" priority="924"/>
-    <cfRule type="duplicateValues" dxfId="77" priority="925"/>
-    <cfRule type="duplicateValues" dxfId="76" priority="926"/>
-    <cfRule type="duplicateValues" dxfId="75" priority="927" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="74" priority="928" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="928" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="927" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="926"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="924"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="923"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="922"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="921"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="925"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D113">
-    <cfRule type="duplicateValues" dxfId="73" priority="53"/>
-    <cfRule type="duplicateValues" dxfId="72" priority="54"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="55" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="70" priority="56" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="57" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="57" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="56" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="55" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D114:D123 D110:D112">
-    <cfRule type="duplicateValues" dxfId="68" priority="58"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="59" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="60"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="61" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="61" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="59" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D119:D122">
-    <cfRule type="duplicateValues" dxfId="64" priority="52" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="52" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D124:D125">
-    <cfRule type="duplicateValues" dxfId="63" priority="47"/>
-    <cfRule type="duplicateValues" dxfId="62" priority="48"/>
-    <cfRule type="duplicateValues" dxfId="61" priority="49" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="50" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="51" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="50" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="51" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="49" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D126">
-    <cfRule type="duplicateValues" dxfId="58" priority="42"/>
-    <cfRule type="duplicateValues" dxfId="57" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="44" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="45" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="46" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="46" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="44" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="45" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D127">
-    <cfRule type="duplicateValues" dxfId="53" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D129">
-    <cfRule type="duplicateValues" dxfId="52" priority="33"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="34"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="35"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="47" priority="38"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="39" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="40" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="39" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="40" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D130">
-    <cfRule type="duplicateValues" dxfId="44" priority="25"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="27"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="28"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="31" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="32" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="32" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="31" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D131">
-    <cfRule type="duplicateValues" dxfId="36" priority="17"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="21"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="22"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="23" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="24" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="24" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="23" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D133:D141">
+    <cfRule type="duplicateValues" dxfId="15" priority="929"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="930"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="931"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="932"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="933"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="934"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="935" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="936" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="28" priority="906"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="907" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1002"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1003" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="26" priority="854"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="855" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="854"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="855" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I67:I73">
-    <cfRule type="duplicateValues" dxfId="24" priority="105"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="105"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="23" priority="852"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="853" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D133:D141">
-    <cfRule type="duplicateValues" dxfId="21" priority="929"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="930"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="931"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="932"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="933"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="934"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="935" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="936" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A44:A66">
-    <cfRule type="duplicateValues" dxfId="13" priority="945"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="946"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D29:D32">
-    <cfRule type="duplicateValues" dxfId="11" priority="949"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="950"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="951"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="952"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="953"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="954"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="955" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="956" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A33:A43">
-    <cfRule type="duplicateValues" dxfId="3" priority="969"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17 D5:D15">
-    <cfRule type="duplicateValues" dxfId="2" priority="975"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="976" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A3:A27">
-    <cfRule type="duplicateValues" dxfId="0" priority="1001"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="852"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="853" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>